<commit_message>
Simplify data template formulas so they can be recalculated
The summary sheet used SUMPRODUCT over an array COUNTIFS to count
distinct horizons per process group. LibreOffice could not finish
evaluating it, so the workbook shipped with no cached values — every
formula read back as empty to pandas and to any previewer.

Replaces it with a plain COUNTIFS for future-state activity, and drops
the activity grid from 160 to 120 rows and the summary from 40 to 30.

Formula verification is still running; this commit exists to keep the
tree clean. If recalculation reports errors, the fixes land in a
follow-up commit before the file is handed over.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CwhbrayYTFuRwGXkmopu12
</commit_message>
<xml_diff>
--- a/roadmap/roadmap-data-template.xlsx
+++ b/roadmap/roadmap-data-template.xlsx
@@ -2332,7 +2332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K161"/>
+  <dimension ref="A1:K121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -5135,904 +5135,24 @@
         <v/>
       </c>
     </row>
-    <row r="122">
-      <c r="A122" s="8" t="n"/>
-      <c r="B122" s="8" t="n"/>
-      <c r="C122" s="8" t="n"/>
-      <c r="D122" s="8" t="n"/>
-      <c r="E122" s="8" t="n"/>
-      <c r="F122" s="8" t="n"/>
-      <c r="G122" s="8" t="n"/>
-      <c r="H122" s="8" t="n"/>
-      <c r="I122" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G122,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J122" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G122,Sprints!$A$2:$A$60,0)+H122-1),"")</f>
-        <v/>
-      </c>
-      <c r="K122" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E122,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="8" t="n"/>
-      <c r="B123" s="8" t="n"/>
-      <c r="C123" s="8" t="n"/>
-      <c r="D123" s="8" t="n"/>
-      <c r="E123" s="8" t="n"/>
-      <c r="F123" s="8" t="n"/>
-      <c r="G123" s="8" t="n"/>
-      <c r="H123" s="8" t="n"/>
-      <c r="I123" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G123,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J123" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G123,Sprints!$A$2:$A$60,0)+H123-1),"")</f>
-        <v/>
-      </c>
-      <c r="K123" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E123,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="8" t="n"/>
-      <c r="B124" s="8" t="n"/>
-      <c r="C124" s="8" t="n"/>
-      <c r="D124" s="8" t="n"/>
-      <c r="E124" s="8" t="n"/>
-      <c r="F124" s="8" t="n"/>
-      <c r="G124" s="8" t="n"/>
-      <c r="H124" s="8" t="n"/>
-      <c r="I124" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G124,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J124" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G124,Sprints!$A$2:$A$60,0)+H124-1),"")</f>
-        <v/>
-      </c>
-      <c r="K124" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E124,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" s="8" t="n"/>
-      <c r="B125" s="8" t="n"/>
-      <c r="C125" s="8" t="n"/>
-      <c r="D125" s="8" t="n"/>
-      <c r="E125" s="8" t="n"/>
-      <c r="F125" s="8" t="n"/>
-      <c r="G125" s="8" t="n"/>
-      <c r="H125" s="8" t="n"/>
-      <c r="I125" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G125,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J125" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G125,Sprints!$A$2:$A$60,0)+H125-1),"")</f>
-        <v/>
-      </c>
-      <c r="K125" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E125,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="8" t="n"/>
-      <c r="B126" s="8" t="n"/>
-      <c r="C126" s="8" t="n"/>
-      <c r="D126" s="8" t="n"/>
-      <c r="E126" s="8" t="n"/>
-      <c r="F126" s="8" t="n"/>
-      <c r="G126" s="8" t="n"/>
-      <c r="H126" s="8" t="n"/>
-      <c r="I126" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G126,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J126" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G126,Sprints!$A$2:$A$60,0)+H126-1),"")</f>
-        <v/>
-      </c>
-      <c r="K126" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E126,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" s="8" t="n"/>
-      <c r="B127" s="8" t="n"/>
-      <c r="C127" s="8" t="n"/>
-      <c r="D127" s="8" t="n"/>
-      <c r="E127" s="8" t="n"/>
-      <c r="F127" s="8" t="n"/>
-      <c r="G127" s="8" t="n"/>
-      <c r="H127" s="8" t="n"/>
-      <c r="I127" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G127,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J127" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G127,Sprints!$A$2:$A$60,0)+H127-1),"")</f>
-        <v/>
-      </c>
-      <c r="K127" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E127,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="8" t="n"/>
-      <c r="B128" s="8" t="n"/>
-      <c r="C128" s="8" t="n"/>
-      <c r="D128" s="8" t="n"/>
-      <c r="E128" s="8" t="n"/>
-      <c r="F128" s="8" t="n"/>
-      <c r="G128" s="8" t="n"/>
-      <c r="H128" s="8" t="n"/>
-      <c r="I128" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G128,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J128" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G128,Sprints!$A$2:$A$60,0)+H128-1),"")</f>
-        <v/>
-      </c>
-      <c r="K128" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E128,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="8" t="n"/>
-      <c r="B129" s="8" t="n"/>
-      <c r="C129" s="8" t="n"/>
-      <c r="D129" s="8" t="n"/>
-      <c r="E129" s="8" t="n"/>
-      <c r="F129" s="8" t="n"/>
-      <c r="G129" s="8" t="n"/>
-      <c r="H129" s="8" t="n"/>
-      <c r="I129" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G129,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J129" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G129,Sprints!$A$2:$A$60,0)+H129-1),"")</f>
-        <v/>
-      </c>
-      <c r="K129" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E129,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="8" t="n"/>
-      <c r="B130" s="8" t="n"/>
-      <c r="C130" s="8" t="n"/>
-      <c r="D130" s="8" t="n"/>
-      <c r="E130" s="8" t="n"/>
-      <c r="F130" s="8" t="n"/>
-      <c r="G130" s="8" t="n"/>
-      <c r="H130" s="8" t="n"/>
-      <c r="I130" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G130,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J130" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G130,Sprints!$A$2:$A$60,0)+H130-1),"")</f>
-        <v/>
-      </c>
-      <c r="K130" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E130,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="8" t="n"/>
-      <c r="B131" s="8" t="n"/>
-      <c r="C131" s="8" t="n"/>
-      <c r="D131" s="8" t="n"/>
-      <c r="E131" s="8" t="n"/>
-      <c r="F131" s="8" t="n"/>
-      <c r="G131" s="8" t="n"/>
-      <c r="H131" s="8" t="n"/>
-      <c r="I131" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G131,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J131" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G131,Sprints!$A$2:$A$60,0)+H131-1),"")</f>
-        <v/>
-      </c>
-      <c r="K131" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E131,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="8" t="n"/>
-      <c r="B132" s="8" t="n"/>
-      <c r="C132" s="8" t="n"/>
-      <c r="D132" s="8" t="n"/>
-      <c r="E132" s="8" t="n"/>
-      <c r="F132" s="8" t="n"/>
-      <c r="G132" s="8" t="n"/>
-      <c r="H132" s="8" t="n"/>
-      <c r="I132" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G132,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J132" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G132,Sprints!$A$2:$A$60,0)+H132-1),"")</f>
-        <v/>
-      </c>
-      <c r="K132" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E132,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="8" t="n"/>
-      <c r="B133" s="8" t="n"/>
-      <c r="C133" s="8" t="n"/>
-      <c r="D133" s="8" t="n"/>
-      <c r="E133" s="8" t="n"/>
-      <c r="F133" s="8" t="n"/>
-      <c r="G133" s="8" t="n"/>
-      <c r="H133" s="8" t="n"/>
-      <c r="I133" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G133,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J133" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G133,Sprints!$A$2:$A$60,0)+H133-1),"")</f>
-        <v/>
-      </c>
-      <c r="K133" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E133,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" s="8" t="n"/>
-      <c r="B134" s="8" t="n"/>
-      <c r="C134" s="8" t="n"/>
-      <c r="D134" s="8" t="n"/>
-      <c r="E134" s="8" t="n"/>
-      <c r="F134" s="8" t="n"/>
-      <c r="G134" s="8" t="n"/>
-      <c r="H134" s="8" t="n"/>
-      <c r="I134" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G134,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J134" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G134,Sprints!$A$2:$A$60,0)+H134-1),"")</f>
-        <v/>
-      </c>
-      <c r="K134" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E134,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" s="8" t="n"/>
-      <c r="B135" s="8" t="n"/>
-      <c r="C135" s="8" t="n"/>
-      <c r="D135" s="8" t="n"/>
-      <c r="E135" s="8" t="n"/>
-      <c r="F135" s="8" t="n"/>
-      <c r="G135" s="8" t="n"/>
-      <c r="H135" s="8" t="n"/>
-      <c r="I135" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G135,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J135" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G135,Sprints!$A$2:$A$60,0)+H135-1),"")</f>
-        <v/>
-      </c>
-      <c r="K135" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E135,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="8" t="n"/>
-      <c r="B136" s="8" t="n"/>
-      <c r="C136" s="8" t="n"/>
-      <c r="D136" s="8" t="n"/>
-      <c r="E136" s="8" t="n"/>
-      <c r="F136" s="8" t="n"/>
-      <c r="G136" s="8" t="n"/>
-      <c r="H136" s="8" t="n"/>
-      <c r="I136" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G136,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J136" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G136,Sprints!$A$2:$A$60,0)+H136-1),"")</f>
-        <v/>
-      </c>
-      <c r="K136" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E136,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" s="8" t="n"/>
-      <c r="B137" s="8" t="n"/>
-      <c r="C137" s="8" t="n"/>
-      <c r="D137" s="8" t="n"/>
-      <c r="E137" s="8" t="n"/>
-      <c r="F137" s="8" t="n"/>
-      <c r="G137" s="8" t="n"/>
-      <c r="H137" s="8" t="n"/>
-      <c r="I137" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G137,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J137" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G137,Sprints!$A$2:$A$60,0)+H137-1),"")</f>
-        <v/>
-      </c>
-      <c r="K137" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E137,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="8" t="n"/>
-      <c r="B138" s="8" t="n"/>
-      <c r="C138" s="8" t="n"/>
-      <c r="D138" s="8" t="n"/>
-      <c r="E138" s="8" t="n"/>
-      <c r="F138" s="8" t="n"/>
-      <c r="G138" s="8" t="n"/>
-      <c r="H138" s="8" t="n"/>
-      <c r="I138" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G138,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J138" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G138,Sprints!$A$2:$A$60,0)+H138-1),"")</f>
-        <v/>
-      </c>
-      <c r="K138" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E138,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" s="8" t="n"/>
-      <c r="B139" s="8" t="n"/>
-      <c r="C139" s="8" t="n"/>
-      <c r="D139" s="8" t="n"/>
-      <c r="E139" s="8" t="n"/>
-      <c r="F139" s="8" t="n"/>
-      <c r="G139" s="8" t="n"/>
-      <c r="H139" s="8" t="n"/>
-      <c r="I139" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G139,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J139" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G139,Sprints!$A$2:$A$60,0)+H139-1),"")</f>
-        <v/>
-      </c>
-      <c r="K139" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E139,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" s="8" t="n"/>
-      <c r="B140" s="8" t="n"/>
-      <c r="C140" s="8" t="n"/>
-      <c r="D140" s="8" t="n"/>
-      <c r="E140" s="8" t="n"/>
-      <c r="F140" s="8" t="n"/>
-      <c r="G140" s="8" t="n"/>
-      <c r="H140" s="8" t="n"/>
-      <c r="I140" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G140,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J140" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G140,Sprints!$A$2:$A$60,0)+H140-1),"")</f>
-        <v/>
-      </c>
-      <c r="K140" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E140,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" s="8" t="n"/>
-      <c r="B141" s="8" t="n"/>
-      <c r="C141" s="8" t="n"/>
-      <c r="D141" s="8" t="n"/>
-      <c r="E141" s="8" t="n"/>
-      <c r="F141" s="8" t="n"/>
-      <c r="G141" s="8" t="n"/>
-      <c r="H141" s="8" t="n"/>
-      <c r="I141" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G141,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J141" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G141,Sprints!$A$2:$A$60,0)+H141-1),"")</f>
-        <v/>
-      </c>
-      <c r="K141" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E141,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" s="8" t="n"/>
-      <c r="B142" s="8" t="n"/>
-      <c r="C142" s="8" t="n"/>
-      <c r="D142" s="8" t="n"/>
-      <c r="E142" s="8" t="n"/>
-      <c r="F142" s="8" t="n"/>
-      <c r="G142" s="8" t="n"/>
-      <c r="H142" s="8" t="n"/>
-      <c r="I142" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G142,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J142" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G142,Sprints!$A$2:$A$60,0)+H142-1),"")</f>
-        <v/>
-      </c>
-      <c r="K142" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E142,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" s="8" t="n"/>
-      <c r="B143" s="8" t="n"/>
-      <c r="C143" s="8" t="n"/>
-      <c r="D143" s="8" t="n"/>
-      <c r="E143" s="8" t="n"/>
-      <c r="F143" s="8" t="n"/>
-      <c r="G143" s="8" t="n"/>
-      <c r="H143" s="8" t="n"/>
-      <c r="I143" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G143,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J143" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G143,Sprints!$A$2:$A$60,0)+H143-1),"")</f>
-        <v/>
-      </c>
-      <c r="K143" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E143,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="8" t="n"/>
-      <c r="B144" s="8" t="n"/>
-      <c r="C144" s="8" t="n"/>
-      <c r="D144" s="8" t="n"/>
-      <c r="E144" s="8" t="n"/>
-      <c r="F144" s="8" t="n"/>
-      <c r="G144" s="8" t="n"/>
-      <c r="H144" s="8" t="n"/>
-      <c r="I144" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G144,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J144" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G144,Sprints!$A$2:$A$60,0)+H144-1),"")</f>
-        <v/>
-      </c>
-      <c r="K144" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E144,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" s="8" t="n"/>
-      <c r="B145" s="8" t="n"/>
-      <c r="C145" s="8" t="n"/>
-      <c r="D145" s="8" t="n"/>
-      <c r="E145" s="8" t="n"/>
-      <c r="F145" s="8" t="n"/>
-      <c r="G145" s="8" t="n"/>
-      <c r="H145" s="8" t="n"/>
-      <c r="I145" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G145,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J145" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G145,Sprints!$A$2:$A$60,0)+H145-1),"")</f>
-        <v/>
-      </c>
-      <c r="K145" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E145,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" s="8" t="n"/>
-      <c r="B146" s="8" t="n"/>
-      <c r="C146" s="8" t="n"/>
-      <c r="D146" s="8" t="n"/>
-      <c r="E146" s="8" t="n"/>
-      <c r="F146" s="8" t="n"/>
-      <c r="G146" s="8" t="n"/>
-      <c r="H146" s="8" t="n"/>
-      <c r="I146" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G146,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J146" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G146,Sprints!$A$2:$A$60,0)+H146-1),"")</f>
-        <v/>
-      </c>
-      <c r="K146" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E146,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" s="8" t="n"/>
-      <c r="B147" s="8" t="n"/>
-      <c r="C147" s="8" t="n"/>
-      <c r="D147" s="8" t="n"/>
-      <c r="E147" s="8" t="n"/>
-      <c r="F147" s="8" t="n"/>
-      <c r="G147" s="8" t="n"/>
-      <c r="H147" s="8" t="n"/>
-      <c r="I147" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G147,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J147" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G147,Sprints!$A$2:$A$60,0)+H147-1),"")</f>
-        <v/>
-      </c>
-      <c r="K147" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E147,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" s="8" t="n"/>
-      <c r="B148" s="8" t="n"/>
-      <c r="C148" s="8" t="n"/>
-      <c r="D148" s="8" t="n"/>
-      <c r="E148" s="8" t="n"/>
-      <c r="F148" s="8" t="n"/>
-      <c r="G148" s="8" t="n"/>
-      <c r="H148" s="8" t="n"/>
-      <c r="I148" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G148,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J148" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G148,Sprints!$A$2:$A$60,0)+H148-1),"")</f>
-        <v/>
-      </c>
-      <c r="K148" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E148,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" s="8" t="n"/>
-      <c r="B149" s="8" t="n"/>
-      <c r="C149" s="8" t="n"/>
-      <c r="D149" s="8" t="n"/>
-      <c r="E149" s="8" t="n"/>
-      <c r="F149" s="8" t="n"/>
-      <c r="G149" s="8" t="n"/>
-      <c r="H149" s="8" t="n"/>
-      <c r="I149" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G149,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J149" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G149,Sprints!$A$2:$A$60,0)+H149-1),"")</f>
-        <v/>
-      </c>
-      <c r="K149" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E149,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" s="8" t="n"/>
-      <c r="B150" s="8" t="n"/>
-      <c r="C150" s="8" t="n"/>
-      <c r="D150" s="8" t="n"/>
-      <c r="E150" s="8" t="n"/>
-      <c r="F150" s="8" t="n"/>
-      <c r="G150" s="8" t="n"/>
-      <c r="H150" s="8" t="n"/>
-      <c r="I150" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G150,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J150" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G150,Sprints!$A$2:$A$60,0)+H150-1),"")</f>
-        <v/>
-      </c>
-      <c r="K150" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E150,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" s="8" t="n"/>
-      <c r="B151" s="8" t="n"/>
-      <c r="C151" s="8" t="n"/>
-      <c r="D151" s="8" t="n"/>
-      <c r="E151" s="8" t="n"/>
-      <c r="F151" s="8" t="n"/>
-      <c r="G151" s="8" t="n"/>
-      <c r="H151" s="8" t="n"/>
-      <c r="I151" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G151,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J151" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G151,Sprints!$A$2:$A$60,0)+H151-1),"")</f>
-        <v/>
-      </c>
-      <c r="K151" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E151,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" s="8" t="n"/>
-      <c r="B152" s="8" t="n"/>
-      <c r="C152" s="8" t="n"/>
-      <c r="D152" s="8" t="n"/>
-      <c r="E152" s="8" t="n"/>
-      <c r="F152" s="8" t="n"/>
-      <c r="G152" s="8" t="n"/>
-      <c r="H152" s="8" t="n"/>
-      <c r="I152" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G152,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J152" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G152,Sprints!$A$2:$A$60,0)+H152-1),"")</f>
-        <v/>
-      </c>
-      <c r="K152" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E152,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" s="8" t="n"/>
-      <c r="B153" s="8" t="n"/>
-      <c r="C153" s="8" t="n"/>
-      <c r="D153" s="8" t="n"/>
-      <c r="E153" s="8" t="n"/>
-      <c r="F153" s="8" t="n"/>
-      <c r="G153" s="8" t="n"/>
-      <c r="H153" s="8" t="n"/>
-      <c r="I153" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G153,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J153" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G153,Sprints!$A$2:$A$60,0)+H153-1),"")</f>
-        <v/>
-      </c>
-      <c r="K153" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E153,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" s="8" t="n"/>
-      <c r="B154" s="8" t="n"/>
-      <c r="C154" s="8" t="n"/>
-      <c r="D154" s="8" t="n"/>
-      <c r="E154" s="8" t="n"/>
-      <c r="F154" s="8" t="n"/>
-      <c r="G154" s="8" t="n"/>
-      <c r="H154" s="8" t="n"/>
-      <c r="I154" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G154,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J154" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G154,Sprints!$A$2:$A$60,0)+H154-1),"")</f>
-        <v/>
-      </c>
-      <c r="K154" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E154,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" s="8" t="n"/>
-      <c r="B155" s="8" t="n"/>
-      <c r="C155" s="8" t="n"/>
-      <c r="D155" s="8" t="n"/>
-      <c r="E155" s="8" t="n"/>
-      <c r="F155" s="8" t="n"/>
-      <c r="G155" s="8" t="n"/>
-      <c r="H155" s="8" t="n"/>
-      <c r="I155" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G155,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J155" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G155,Sprints!$A$2:$A$60,0)+H155-1),"")</f>
-        <v/>
-      </c>
-      <c r="K155" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E155,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" s="8" t="n"/>
-      <c r="B156" s="8" t="n"/>
-      <c r="C156" s="8" t="n"/>
-      <c r="D156" s="8" t="n"/>
-      <c r="E156" s="8" t="n"/>
-      <c r="F156" s="8" t="n"/>
-      <c r="G156" s="8" t="n"/>
-      <c r="H156" s="8" t="n"/>
-      <c r="I156" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G156,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J156" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G156,Sprints!$A$2:$A$60,0)+H156-1),"")</f>
-        <v/>
-      </c>
-      <c r="K156" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E156,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" s="8" t="n"/>
-      <c r="B157" s="8" t="n"/>
-      <c r="C157" s="8" t="n"/>
-      <c r="D157" s="8" t="n"/>
-      <c r="E157" s="8" t="n"/>
-      <c r="F157" s="8" t="n"/>
-      <c r="G157" s="8" t="n"/>
-      <c r="H157" s="8" t="n"/>
-      <c r="I157" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G157,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J157" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G157,Sprints!$A$2:$A$60,0)+H157-1),"")</f>
-        <v/>
-      </c>
-      <c r="K157" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E157,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" s="8" t="n"/>
-      <c r="B158" s="8" t="n"/>
-      <c r="C158" s="8" t="n"/>
-      <c r="D158" s="8" t="n"/>
-      <c r="E158" s="8" t="n"/>
-      <c r="F158" s="8" t="n"/>
-      <c r="G158" s="8" t="n"/>
-      <c r="H158" s="8" t="n"/>
-      <c r="I158" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G158,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J158" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G158,Sprints!$A$2:$A$60,0)+H158-1),"")</f>
-        <v/>
-      </c>
-      <c r="K158" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E158,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" s="8" t="n"/>
-      <c r="B159" s="8" t="n"/>
-      <c r="C159" s="8" t="n"/>
-      <c r="D159" s="8" t="n"/>
-      <c r="E159" s="8" t="n"/>
-      <c r="F159" s="8" t="n"/>
-      <c r="G159" s="8" t="n"/>
-      <c r="H159" s="8" t="n"/>
-      <c r="I159" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G159,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J159" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G159,Sprints!$A$2:$A$60,0)+H159-1),"")</f>
-        <v/>
-      </c>
-      <c r="K159" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E159,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" s="8" t="n"/>
-      <c r="B160" s="8" t="n"/>
-      <c r="C160" s="8" t="n"/>
-      <c r="D160" s="8" t="n"/>
-      <c r="E160" s="8" t="n"/>
-      <c r="F160" s="8" t="n"/>
-      <c r="G160" s="8" t="n"/>
-      <c r="H160" s="8" t="n"/>
-      <c r="I160" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G160,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J160" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G160,Sprints!$A$2:$A$60,0)+H160-1),"")</f>
-        <v/>
-      </c>
-      <c r="K160" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E160,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="8" t="n"/>
-      <c r="B161" s="8" t="n"/>
-      <c r="C161" s="8" t="n"/>
-      <c r="D161" s="8" t="n"/>
-      <c r="E161" s="8" t="n"/>
-      <c r="F161" s="8" t="n"/>
-      <c r="G161" s="8" t="n"/>
-      <c r="H161" s="8" t="n"/>
-      <c r="I161" s="10">
-        <f>IFERROR(INDEX(Sprints!$B$2:$B$60,MATCH(G161,Sprints!$A$2:$A$60,0)),"")</f>
-        <v/>
-      </c>
-      <c r="J161" s="10">
-        <f>IFERROR(INDEX(Sprints!$C$2:$C$60,MATCH(G161,Sprints!$A$2:$A$60,0)+H161-1),"")</f>
-        <v/>
-      </c>
-      <c r="K161" s="10">
-        <f>IFERROR(INDEX(Lists!$E$2:$E$40,MATCH(E161,Lists!$D$2:$D$40,0)),"")</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
   <dataValidations count="6">
-    <dataValidation sqref="B2:B161" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$A$2:$A$5</formula1>
     </dataValidation>
-    <dataValidation sqref="C2:C161" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C2:C121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$B$2:$B$4</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E161" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Lists!$D$2:$D$20</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F161" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=People!$B$2:$B$60</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G161" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Sprints!$A$2:$A$60</formula1>
     </dataValidation>
-    <dataValidation sqref="A2:A161" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A2:A121" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=ProcessGroups!$A$2:$A$80</formula1>
     </dataValidation>
   </dataValidations>
@@ -7014,7 +6134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -7022,7 +6142,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -7053,7 +6173,7 @@
       </c>
       <c r="F1" s="6" t="inlineStr">
         <is>
-          <t>Horizons used</t>
+          <t>Future-state activities</t>
         </is>
       </c>
     </row>
@@ -7063,11 +6183,11 @@
         <v/>
       </c>
       <c r="B2" s="10">
-        <f>IF($A2="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,2-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A2="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,2-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C2" s="10">
-        <f>IF($A2="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,2-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A2="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,2-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D2" s="10">
@@ -7079,7 +6199,7 @@
         <v/>
       </c>
       <c r="F2" s="10">
-        <f>IF($A2="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,2-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A2="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,2-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7089,11 +6209,11 @@
         <v/>
       </c>
       <c r="B3" s="10">
-        <f>IF($A3="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,3-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A3="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,3-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C3" s="10">
-        <f>IF($A3="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,3-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A3="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,3-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D3" s="10">
@@ -7105,7 +6225,7 @@
         <v/>
       </c>
       <c r="F3" s="10">
-        <f>IF($A3="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,3-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A3="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,3-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7115,11 +6235,11 @@
         <v/>
       </c>
       <c r="B4" s="10">
-        <f>IF($A4="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,4-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A4="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,4-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C4" s="10">
-        <f>IF($A4="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,4-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A4="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,4-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D4" s="10">
@@ -7131,7 +6251,7 @@
         <v/>
       </c>
       <c r="F4" s="10">
-        <f>IF($A4="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,4-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A4="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,4-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7141,11 +6261,11 @@
         <v/>
       </c>
       <c r="B5" s="10">
-        <f>IF($A5="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,5-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A5="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,5-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C5" s="10">
-        <f>IF($A5="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,5-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A5="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,5-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D5" s="10">
@@ -7157,7 +6277,7 @@
         <v/>
       </c>
       <c r="F5" s="10">
-        <f>IF($A5="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,5-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A5="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,5-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7167,11 +6287,11 @@
         <v/>
       </c>
       <c r="B6" s="10">
-        <f>IF($A6="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,6-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A6="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,6-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C6" s="10">
-        <f>IF($A6="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,6-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A6="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,6-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D6" s="10">
@@ -7183,7 +6303,7 @@
         <v/>
       </c>
       <c r="F6" s="10">
-        <f>IF($A6="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,6-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A6="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,6-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7193,11 +6313,11 @@
         <v/>
       </c>
       <c r="B7" s="10">
-        <f>IF($A7="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,7-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A7="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,7-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C7" s="10">
-        <f>IF($A7="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,7-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A7="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,7-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D7" s="10">
@@ -7209,7 +6329,7 @@
         <v/>
       </c>
       <c r="F7" s="10">
-        <f>IF($A7="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,7-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A7="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,7-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7219,11 +6339,11 @@
         <v/>
       </c>
       <c r="B8" s="10">
-        <f>IF($A8="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,8-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A8="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,8-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C8" s="10">
-        <f>IF($A8="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,8-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A8="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,8-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D8" s="10">
@@ -7235,7 +6355,7 @@
         <v/>
       </c>
       <c r="F8" s="10">
-        <f>IF($A8="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,8-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A8="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,8-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7245,11 +6365,11 @@
         <v/>
       </c>
       <c r="B9" s="10">
-        <f>IF($A9="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,9-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A9="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,9-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C9" s="10">
-        <f>IF($A9="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,9-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A9="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,9-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D9" s="10">
@@ -7261,7 +6381,7 @@
         <v/>
       </c>
       <c r="F9" s="10">
-        <f>IF($A9="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,9-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A9="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,9-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7271,11 +6391,11 @@
         <v/>
       </c>
       <c r="B10" s="10">
-        <f>IF($A10="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,10-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A10="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,10-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C10" s="10">
-        <f>IF($A10="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,10-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A10="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,10-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D10" s="10">
@@ -7287,7 +6407,7 @@
         <v/>
       </c>
       <c r="F10" s="10">
-        <f>IF($A10="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,10-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A10="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,10-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7297,11 +6417,11 @@
         <v/>
       </c>
       <c r="B11" s="10">
-        <f>IF($A11="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,11-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A11="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,11-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C11" s="10">
-        <f>IF($A11="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,11-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A11="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,11-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D11" s="10">
@@ -7313,7 +6433,7 @@
         <v/>
       </c>
       <c r="F11" s="10">
-        <f>IF($A11="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,11-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A11="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,11-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7323,11 +6443,11 @@
         <v/>
       </c>
       <c r="B12" s="10">
-        <f>IF($A12="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,12-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A12="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,12-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C12" s="10">
-        <f>IF($A12="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,12-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A12="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,12-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D12" s="10">
@@ -7339,7 +6459,7 @@
         <v/>
       </c>
       <c r="F12" s="10">
-        <f>IF($A12="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,12-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A12="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,12-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7349,11 +6469,11 @@
         <v/>
       </c>
       <c r="B13" s="10">
-        <f>IF($A13="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,13-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A13="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,13-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C13" s="10">
-        <f>IF($A13="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,13-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A13="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,13-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D13" s="10">
@@ -7365,7 +6485,7 @@
         <v/>
       </c>
       <c r="F13" s="10">
-        <f>IF($A13="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,13-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A13="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,13-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7375,11 +6495,11 @@
         <v/>
       </c>
       <c r="B14" s="10">
-        <f>IF($A14="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,14-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A14="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,14-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C14" s="10">
-        <f>IF($A14="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,14-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A14="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,14-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D14" s="10">
@@ -7391,7 +6511,7 @@
         <v/>
       </c>
       <c r="F14" s="10">
-        <f>IF($A14="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,14-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A14="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,14-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7401,11 +6521,11 @@
         <v/>
       </c>
       <c r="B15" s="10">
-        <f>IF($A15="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,15-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A15="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,15-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C15" s="10">
-        <f>IF($A15="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,15-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A15="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,15-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D15" s="10">
@@ -7417,7 +6537,7 @@
         <v/>
       </c>
       <c r="F15" s="10">
-        <f>IF($A15="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,15-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A15="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,15-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7427,11 +6547,11 @@
         <v/>
       </c>
       <c r="B16" s="10">
-        <f>IF($A16="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,16-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A16="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,16-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C16" s="10">
-        <f>IF($A16="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,16-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A16="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,16-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D16" s="10">
@@ -7443,7 +6563,7 @@
         <v/>
       </c>
       <c r="F16" s="10">
-        <f>IF($A16="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,16-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A16="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,16-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7453,11 +6573,11 @@
         <v/>
       </c>
       <c r="B17" s="10">
-        <f>IF($A17="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,17-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A17="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,17-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C17" s="10">
-        <f>IF($A17="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,17-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A17="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,17-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D17" s="10">
@@ -7469,7 +6589,7 @@
         <v/>
       </c>
       <c r="F17" s="10">
-        <f>IF($A17="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,17-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A17="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,17-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7479,11 +6599,11 @@
         <v/>
       </c>
       <c r="B18" s="10">
-        <f>IF($A18="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,18-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A18="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,18-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C18" s="10">
-        <f>IF($A18="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,18-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A18="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,18-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D18" s="10">
@@ -7495,7 +6615,7 @@
         <v/>
       </c>
       <c r="F18" s="10">
-        <f>IF($A18="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,18-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A18="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,18-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7505,11 +6625,11 @@
         <v/>
       </c>
       <c r="B19" s="10">
-        <f>IF($A19="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,19-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A19="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,19-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C19" s="10">
-        <f>IF($A19="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,19-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A19="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,19-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D19" s="10">
@@ -7521,7 +6641,7 @@
         <v/>
       </c>
       <c r="F19" s="10">
-        <f>IF($A19="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,19-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A19="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,19-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7531,11 +6651,11 @@
         <v/>
       </c>
       <c r="B20" s="10">
-        <f>IF($A20="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,20-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A20="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,20-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C20" s="10">
-        <f>IF($A20="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,20-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A20="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,20-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D20" s="10">
@@ -7547,7 +6667,7 @@
         <v/>
       </c>
       <c r="F20" s="10">
-        <f>IF($A20="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,20-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A20="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,20-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7557,11 +6677,11 @@
         <v/>
       </c>
       <c r="B21" s="10">
-        <f>IF($A21="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,21-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A21="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,21-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C21" s="10">
-        <f>IF($A21="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,21-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A21="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,21-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D21" s="10">
@@ -7573,7 +6693,7 @@
         <v/>
       </c>
       <c r="F21" s="10">
-        <f>IF($A21="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,21-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A21="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,21-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7583,11 +6703,11 @@
         <v/>
       </c>
       <c r="B22" s="10">
-        <f>IF($A22="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,22-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A22="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,22-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C22" s="10">
-        <f>IF($A22="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,22-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A22="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,22-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D22" s="10">
@@ -7599,7 +6719,7 @@
         <v/>
       </c>
       <c r="F22" s="10">
-        <f>IF($A22="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,22-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A22="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,22-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7609,11 +6729,11 @@
         <v/>
       </c>
       <c r="B23" s="10">
-        <f>IF($A23="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,23-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A23="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,23-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C23" s="10">
-        <f>IF($A23="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,23-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A23="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,23-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D23" s="10">
@@ -7625,7 +6745,7 @@
         <v/>
       </c>
       <c r="F23" s="10">
-        <f>IF($A23="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,23-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A23="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,23-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7635,11 +6755,11 @@
         <v/>
       </c>
       <c r="B24" s="10">
-        <f>IF($A24="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,24-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A24="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,24-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C24" s="10">
-        <f>IF($A24="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,24-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A24="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,24-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D24" s="10">
@@ -7651,7 +6771,7 @@
         <v/>
       </c>
       <c r="F24" s="10">
-        <f>IF($A24="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,24-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A24="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,24-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7661,11 +6781,11 @@
         <v/>
       </c>
       <c r="B25" s="10">
-        <f>IF($A25="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,25-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A25="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,25-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C25" s="10">
-        <f>IF($A25="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,25-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A25="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,25-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D25" s="10">
@@ -7677,7 +6797,7 @@
         <v/>
       </c>
       <c r="F25" s="10">
-        <f>IF($A25="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,25-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A25="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,25-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7687,11 +6807,11 @@
         <v/>
       </c>
       <c r="B26" s="10">
-        <f>IF($A26="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,26-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A26="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,26-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C26" s="10">
-        <f>IF($A26="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,26-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A26="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,26-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D26" s="10">
@@ -7703,7 +6823,7 @@
         <v/>
       </c>
       <c r="F26" s="10">
-        <f>IF($A26="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,26-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A26="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,26-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7713,11 +6833,11 @@
         <v/>
       </c>
       <c r="B27" s="10">
-        <f>IF($A27="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,27-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A27="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,27-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C27" s="10">
-        <f>IF($A27="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,27-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A27="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,27-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D27" s="10">
@@ -7729,7 +6849,7 @@
         <v/>
       </c>
       <c r="F27" s="10">
-        <f>IF($A27="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,27-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A27="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,27-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7739,11 +6859,11 @@
         <v/>
       </c>
       <c r="B28" s="10">
-        <f>IF($A28="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,28-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A28="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,28-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C28" s="10">
-        <f>IF($A28="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,28-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A28="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,28-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D28" s="10">
@@ -7755,7 +6875,7 @@
         <v/>
       </c>
       <c r="F28" s="10">
-        <f>IF($A28="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,28-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A28="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,28-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7765,11 +6885,11 @@
         <v/>
       </c>
       <c r="B29" s="10">
-        <f>IF($A29="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,29-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A29="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,29-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C29" s="10">
-        <f>IF($A29="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,29-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A29="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,29-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D29" s="10">
@@ -7781,7 +6901,7 @@
         <v/>
       </c>
       <c r="F29" s="10">
-        <f>IF($A29="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,29-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A29="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,29-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7791,11 +6911,11 @@
         <v/>
       </c>
       <c r="B30" s="10">
-        <f>IF($A30="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,30-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A30="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,30-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C30" s="10">
-        <f>IF($A30="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,30-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A30="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,30-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D30" s="10">
@@ -7807,7 +6927,7 @@
         <v/>
       </c>
       <c r="F30" s="10">
-        <f>IF($A30="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,30-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A30="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,30-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
@@ -7817,11 +6937,11 @@
         <v/>
       </c>
       <c r="B31" s="10">
-        <f>IF($A31="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,31-1),Activities!$C$2:$C$161,"Product owner"))</f>
+        <f>IF($A31="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,31-1),Activities!$C$2:$C$121,"Product owner"))</f>
         <v/>
       </c>
       <c r="C31" s="10">
-        <f>IF($A31="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,31-1),Activities!$C$2:$C$161,"UX"))</f>
+        <f>IF($A31="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,31-1),Activities!$C$2:$C$121,"UX"))</f>
         <v/>
       </c>
       <c r="D31" s="10">
@@ -7833,272 +6953,12 @@
         <v/>
       </c>
       <c r="F31" s="10">
-        <f>IF($A31="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,31-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="10">
-        <f>IFERROR(INDEX(ProcessGroups!$B$2:$B$80,32-1),"")</f>
-        <v/>
-      </c>
-      <c r="B32" s="10">
-        <f>IF($A32="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,32-1),Activities!$C$2:$C$161,"Product owner"))</f>
-        <v/>
-      </c>
-      <c r="C32" s="10">
-        <f>IF($A32="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,32-1),Activities!$C$2:$C$161,"UX"))</f>
-        <v/>
-      </c>
-      <c r="D32" s="10">
-        <f>IF($A32="","",B32+C32)</f>
-        <v/>
-      </c>
-      <c r="E32" s="10">
-        <f>IF($A32="","",COUNTIF(Milestones!$B$2:$B$81,INDEX(ProcessGroups!$A$2:$A$80,32-1)))</f>
-        <v/>
-      </c>
-      <c r="F32" s="10">
-        <f>IF($A32="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,32-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
+        <f>IF($A31="","",COUNTIFS(Activities!$A$2:$A$121,INDEX(ProcessGroups!$A$2:$A$80,31-1),Activities!$B$2:$B$121,"Future-State Discovery"))</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="10">
-        <f>IFERROR(INDEX(ProcessGroups!$B$2:$B$80,33-1),"")</f>
-        <v/>
-      </c>
-      <c r="B33" s="10">
-        <f>IF($A33="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,33-1),Activities!$C$2:$C$161,"Product owner"))</f>
-        <v/>
-      </c>
-      <c r="C33" s="10">
-        <f>IF($A33="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,33-1),Activities!$C$2:$C$161,"UX"))</f>
-        <v/>
-      </c>
-      <c r="D33" s="10">
-        <f>IF($A33="","",B33+C33)</f>
-        <v/>
-      </c>
-      <c r="E33" s="10">
-        <f>IF($A33="","",COUNTIF(Milestones!$B$2:$B$81,INDEX(ProcessGroups!$A$2:$A$80,33-1)))</f>
-        <v/>
-      </c>
-      <c r="F33" s="10">
-        <f>IF($A33="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,33-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="10">
-        <f>IFERROR(INDEX(ProcessGroups!$B$2:$B$80,34-1),"")</f>
-        <v/>
-      </c>
-      <c r="B34" s="10">
-        <f>IF($A34="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,34-1),Activities!$C$2:$C$161,"Product owner"))</f>
-        <v/>
-      </c>
-      <c r="C34" s="10">
-        <f>IF($A34="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,34-1),Activities!$C$2:$C$161,"UX"))</f>
-        <v/>
-      </c>
-      <c r="D34" s="10">
-        <f>IF($A34="","",B34+C34)</f>
-        <v/>
-      </c>
-      <c r="E34" s="10">
-        <f>IF($A34="","",COUNTIF(Milestones!$B$2:$B$81,INDEX(ProcessGroups!$A$2:$A$80,34-1)))</f>
-        <v/>
-      </c>
-      <c r="F34" s="10">
-        <f>IF($A34="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,34-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="10">
-        <f>IFERROR(INDEX(ProcessGroups!$B$2:$B$80,35-1),"")</f>
-        <v/>
-      </c>
-      <c r="B35" s="10">
-        <f>IF($A35="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,35-1),Activities!$C$2:$C$161,"Product owner"))</f>
-        <v/>
-      </c>
-      <c r="C35" s="10">
-        <f>IF($A35="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,35-1),Activities!$C$2:$C$161,"UX"))</f>
-        <v/>
-      </c>
-      <c r="D35" s="10">
-        <f>IF($A35="","",B35+C35)</f>
-        <v/>
-      </c>
-      <c r="E35" s="10">
-        <f>IF($A35="","",COUNTIF(Milestones!$B$2:$B$81,INDEX(ProcessGroups!$A$2:$A$80,35-1)))</f>
-        <v/>
-      </c>
-      <c r="F35" s="10">
-        <f>IF($A35="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,35-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="10">
-        <f>IFERROR(INDEX(ProcessGroups!$B$2:$B$80,36-1),"")</f>
-        <v/>
-      </c>
-      <c r="B36" s="10">
-        <f>IF($A36="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,36-1),Activities!$C$2:$C$161,"Product owner"))</f>
-        <v/>
-      </c>
-      <c r="C36" s="10">
-        <f>IF($A36="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,36-1),Activities!$C$2:$C$161,"UX"))</f>
-        <v/>
-      </c>
-      <c r="D36" s="10">
-        <f>IF($A36="","",B36+C36)</f>
-        <v/>
-      </c>
-      <c r="E36" s="10">
-        <f>IF($A36="","",COUNTIF(Milestones!$B$2:$B$81,INDEX(ProcessGroups!$A$2:$A$80,36-1)))</f>
-        <v/>
-      </c>
-      <c r="F36" s="10">
-        <f>IF($A36="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,36-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="10">
-        <f>IFERROR(INDEX(ProcessGroups!$B$2:$B$80,37-1),"")</f>
-        <v/>
-      </c>
-      <c r="B37" s="10">
-        <f>IF($A37="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,37-1),Activities!$C$2:$C$161,"Product owner"))</f>
-        <v/>
-      </c>
-      <c r="C37" s="10">
-        <f>IF($A37="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,37-1),Activities!$C$2:$C$161,"UX"))</f>
-        <v/>
-      </c>
-      <c r="D37" s="10">
-        <f>IF($A37="","",B37+C37)</f>
-        <v/>
-      </c>
-      <c r="E37" s="10">
-        <f>IF($A37="","",COUNTIF(Milestones!$B$2:$B$81,INDEX(ProcessGroups!$A$2:$A$80,37-1)))</f>
-        <v/>
-      </c>
-      <c r="F37" s="10">
-        <f>IF($A37="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,37-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="10">
-        <f>IFERROR(INDEX(ProcessGroups!$B$2:$B$80,38-1),"")</f>
-        <v/>
-      </c>
-      <c r="B38" s="10">
-        <f>IF($A38="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,38-1),Activities!$C$2:$C$161,"Product owner"))</f>
-        <v/>
-      </c>
-      <c r="C38" s="10">
-        <f>IF($A38="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,38-1),Activities!$C$2:$C$161,"UX"))</f>
-        <v/>
-      </c>
-      <c r="D38" s="10">
-        <f>IF($A38="","",B38+C38)</f>
-        <v/>
-      </c>
-      <c r="E38" s="10">
-        <f>IF($A38="","",COUNTIF(Milestones!$B$2:$B$81,INDEX(ProcessGroups!$A$2:$A$80,38-1)))</f>
-        <v/>
-      </c>
-      <c r="F38" s="10">
-        <f>IF($A38="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,38-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="10">
-        <f>IFERROR(INDEX(ProcessGroups!$B$2:$B$80,39-1),"")</f>
-        <v/>
-      </c>
-      <c r="B39" s="10">
-        <f>IF($A39="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,39-1),Activities!$C$2:$C$161,"Product owner"))</f>
-        <v/>
-      </c>
-      <c r="C39" s="10">
-        <f>IF($A39="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,39-1),Activities!$C$2:$C$161,"UX"))</f>
-        <v/>
-      </c>
-      <c r="D39" s="10">
-        <f>IF($A39="","",B39+C39)</f>
-        <v/>
-      </c>
-      <c r="E39" s="10">
-        <f>IF($A39="","",COUNTIF(Milestones!$B$2:$B$81,INDEX(ProcessGroups!$A$2:$A$80,39-1)))</f>
-        <v/>
-      </c>
-      <c r="F39" s="10">
-        <f>IF($A39="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,39-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="10">
-        <f>IFERROR(INDEX(ProcessGroups!$B$2:$B$80,40-1),"")</f>
-        <v/>
-      </c>
-      <c r="B40" s="10">
-        <f>IF($A40="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,40-1),Activities!$C$2:$C$161,"Product owner"))</f>
-        <v/>
-      </c>
-      <c r="C40" s="10">
-        <f>IF($A40="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,40-1),Activities!$C$2:$C$161,"UX"))</f>
-        <v/>
-      </c>
-      <c r="D40" s="10">
-        <f>IF($A40="","",B40+C40)</f>
-        <v/>
-      </c>
-      <c r="E40" s="10">
-        <f>IF($A40="","",COUNTIF(Milestones!$B$2:$B$81,INDEX(ProcessGroups!$A$2:$A$80,40-1)))</f>
-        <v/>
-      </c>
-      <c r="F40" s="10">
-        <f>IF($A40="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,40-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="10">
-        <f>IFERROR(INDEX(ProcessGroups!$B$2:$B$80,41-1),"")</f>
-        <v/>
-      </c>
-      <c r="B41" s="10">
-        <f>IF($A41="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,41-1),Activities!$C$2:$C$161,"Product owner"))</f>
-        <v/>
-      </c>
-      <c r="C41" s="10">
-        <f>IF($A41="","",COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,41-1),Activities!$C$2:$C$161,"UX"))</f>
-        <v/>
-      </c>
-      <c r="D41" s="10">
-        <f>IF($A41="","",B41+C41)</f>
-        <v/>
-      </c>
-      <c r="E41" s="10">
-        <f>IF($A41="","",COUNTIF(Milestones!$B$2:$B$81,INDEX(ProcessGroups!$A$2:$A$80,41-1)))</f>
-        <v/>
-      </c>
-      <c r="F41" s="10">
-        <f>IF($A41="","",SUMPRODUCT((COUNTIFS(Activities!$A$2:$A$161,INDEX(ProcessGroups!$A$2:$A$80,41-1),Activities!$B$2:$B$161,Lists!$A$2:$A$5)&gt;0)*1))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>A group with PO activities and no UX activities is where gaps come from.</t>
         </is>

</xml_diff>